<commit_message>
🔄 auto: 2026-06-26 13:47
</commit_message>
<xml_diff>
--- a/skills/proofread-docx/glossaries/术语库_标准格式.xlsx
+++ b/skills/proofread-docx/glossaries/术语库_标准格式.xlsx
@@ -76302,7 +76302,11 @@
           <t>Ulthera</t>
         </is>
       </c>
-      <c r="B2811" s="4" t="inlineStr"/>
+      <c r="B2811" s="4" t="inlineStr">
+        <is>
+          <t>Ulthera（品牌名，保留不译）</t>
+        </is>
+      </c>
       <c r="C2811" s="5" t="inlineStr">
         <is>
           <t>保留原文</t>
@@ -76315,7 +76319,7 @@
       </c>
       <c r="E2811" s="4" t="inlineStr">
         <is>
-          <t>Phase5查证：Ulthera系统品牌名，保留不译</t>
+          <t>品牌名，保留不译</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 auto: 2026-06-26 15:17
</commit_message>
<xml_diff>
--- a/skills/proofread-docx/glossaries/术语库_标准格式.xlsx
+++ b/skills/proofread-docx/glossaries/术语库_标准格式.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2814"/>
+  <dimension ref="A1:F2814"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -522,6 +522,11 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>入库时间</t>
         </is>
       </c>
     </row>

</xml_diff>